<commit_message>
Woopsies, should have used the cleaned data
</commit_message>
<xml_diff>
--- a/Cell survival results/PH_means.xlsx
+++ b/Cell survival results/PH_means.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -520,190 +520,190 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="B5" t="n">
-        <v>0.007585043818827907</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0.006170483568739783</v>
+        <v>0.5238365618002725</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>EXP_2025_10_16</t>
+          <t>EXP_2025_11_18</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>#00FFFF</t>
+          <t>#00008B</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>0.12150937028843</v>
       </c>
       <c r="C6" t="n">
-        <v>0.5411577928635585</v>
+        <v>0.02436652766184981</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>EXP_2025_10_30</t>
+          <t>EXP_2025_11_18</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>#0000FF</t>
+          <t>#00008B</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>0.4599170581101318</v>
+        <v>0.003775365713321406</v>
       </c>
       <c r="C7" t="n">
-        <v>0.05900074272861982</v>
+        <v>0.0002747779729281328</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EXP_2025_10_30</t>
+          <t>EXP_2025_11_18</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>#0000FF</t>
+          <t>#00008B</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B8" t="n">
-        <v>0.00230451064410692</v>
+        <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0006021679080668702</v>
+        <v>0.08737820577231911</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>EXP_2025_10_30</t>
+          <t>EXP_2026_2_04</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>#0000FF</t>
+          <t>#4B0082</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B9" t="n">
-        <v>0.0003838328190425245</v>
+        <v>0.06116905324329176</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0001736129910497663</v>
+        <v>0.005529857803049707</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EXP_2025_10_30</t>
+          <t>EXP_2026_2_04</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>#0000FF</t>
+          <t>#4B0082</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>0.01067022708838941</v>
       </c>
       <c r="C10" t="n">
-        <v>0.5238365618002725</v>
+        <v>0.00165728377627281</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>EXP_2025_11_18</t>
+          <t>EXP_2026_2_04</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>#00008B</t>
+          <t>#4B0082</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B11" t="n">
-        <v>0.12150937028843</v>
+        <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>0.02436652766184981</v>
+        <v>0.1260936497896067</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>EXP_2025_11_18</t>
+          <t>EXP_2026_2_26</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>#00008B</t>
+          <t>#008080</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B12" t="n">
-        <v>0.003775365713321406</v>
+        <v>0.1951710815889132</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0002747779729281328</v>
+        <v>0.03530291808587505</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EXP_2025_11_18</t>
+          <t>EXP_2026_2_26</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>#00008B</t>
+          <t>#008080</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B13" t="n">
-        <v>0.00278620037221647</v>
+        <v>0.01196557377144132</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0002098123160324973</v>
+        <v>0.002498508881208067</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>EXP_2025_11_18</t>
+          <t>EXP_2026_2_26</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>#00008B</t>
+          <t>#008080</t>
         </is>
       </c>
     </row>
@@ -715,16 +715,16 @@
         <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>0.08737820577231911</v>
+        <v>0.1053728227082863</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>EXP_2026_2_04</t>
+          <t>EXP_2026_3_02</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>#4B0082</t>
+          <t>#FF00FF</t>
         </is>
       </c>
     </row>
@@ -733,19 +733,19 @@
         <v>2</v>
       </c>
       <c r="B15" t="n">
-        <v>0.06116905324329176</v>
+        <v>0.1928145469810209</v>
       </c>
       <c r="C15" t="n">
-        <v>0.005529857803049707</v>
+        <v>0.009854448004505917</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EXP_2026_2_04</t>
+          <t>EXP_2026_3_02</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>#4B0082</t>
+          <t>#FF00FF</t>
         </is>
       </c>
     </row>
@@ -754,374 +754,80 @@
         <v>5</v>
       </c>
       <c r="B16" t="n">
-        <v>0.01067022708838941</v>
+        <v>0.006118341780794272</v>
       </c>
       <c r="C16" t="n">
-        <v>0.00165728377627281</v>
+        <v>0.0006194657575171056</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>EXP_2026_2_04</t>
+          <t>EXP_2026_3_02</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>#4B0082</t>
+          <t>#FF00FF</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="B17" t="n">
-        <v>0.003029859553409619</v>
+        <v>1</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0004231497840487229</v>
+        <v>0.1013460046033881</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>EXP_2026_2_04</t>
+          <t>EXP_2026_3_19</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>#4B0082</t>
+          <t>#00FF00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>0.1932982138393525</v>
       </c>
       <c r="C18" t="n">
-        <v>0.1260936497896067</v>
+        <v>0.01308004534867321</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>EXP_2026_2_26</t>
+          <t>EXP_2026_3_19</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>#008080</t>
+          <t>#00FF00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B19" t="n">
-        <v>0.1951710815889132</v>
+        <v>0.01262775560970711</v>
       </c>
       <c r="C19" t="n">
-        <v>0.03530291808587505</v>
+        <v>0.005459988344673575</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>EXP_2026_2_26</t>
+          <t>EXP_2026_3_19</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
-        <is>
-          <t>#008080</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>5</v>
-      </c>
-      <c r="B20" t="n">
-        <v>0.01196557377144132</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0.002498508881208067</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>EXP_2026_2_26</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>#008080</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>8</v>
-      </c>
-      <c r="B21" t="n">
-        <v>0.0007588037654036302</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0.0005036456302642818</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>EXP_2026_2_26</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>#008080</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>0</v>
-      </c>
-      <c r="B22" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0.1053728227082863</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_02</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>#FF00FF</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>2</v>
-      </c>
-      <c r="B23" t="n">
-        <v>0.1928145469810209</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0.009854448004505917</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_02</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>#FF00FF</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>5</v>
-      </c>
-      <c r="B24" t="n">
-        <v>0.006118341780794272</v>
-      </c>
-      <c r="C24" t="n">
-        <v>0.0006194657575171056</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_02</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>#FF00FF</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>8</v>
-      </c>
-      <c r="B25" t="n">
-        <v>0.0003581340773795413</v>
-      </c>
-      <c r="C25" t="n">
-        <v>0.0003331234283952536</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_02</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>#FF00FF</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>0</v>
-      </c>
-      <c r="B26" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" t="n">
-        <v>1.222952782016584</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_18</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>#008000</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>2</v>
-      </c>
-      <c r="B27" t="n">
-        <v>0.02149691986228468</v>
-      </c>
-      <c r="C27" t="n">
-        <v>0.008802478767641958</v>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_18</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>#008000</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>5</v>
-      </c>
-      <c r="B28" t="n">
-        <v>0.009390821905916997</v>
-      </c>
-      <c r="C28" t="n">
-        <v>0.004026108974519772</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_18</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>#008000</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>8</v>
-      </c>
-      <c r="B29" t="n">
-        <v>0.00299371576458829</v>
-      </c>
-      <c r="C29" t="n">
-        <v>0.001340231051885078</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_18</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>#008000</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>0</v>
-      </c>
-      <c r="B30" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" t="n">
-        <v>0.1013460046033881</v>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_19</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>#00FF00</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>2</v>
-      </c>
-      <c r="B31" t="n">
-        <v>0.1932982138393525</v>
-      </c>
-      <c r="C31" t="n">
-        <v>0.01308004534867321</v>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_19</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>#00FF00</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>5</v>
-      </c>
-      <c r="B32" t="n">
-        <v>0.01262775560970711</v>
-      </c>
-      <c r="C32" t="n">
-        <v>0.005459988344673575</v>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_19</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>#00FF00</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>8</v>
-      </c>
-      <c r="B33" t="n">
-        <v>0.00146626096818678</v>
-      </c>
-      <c r="C33" t="n">
-        <v>0.0008277753700459434</v>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_19</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
         <is>
           <t>#00FF00</t>
         </is>

</xml_diff>